<commit_message>
TAREFA 12 parcialmente concluída
</commit_message>
<xml_diff>
--- a/Avancado/12 - Teste de Hipóteses - Cenários.xlsx
+++ b/Avancado/12 - Teste de Hipóteses - Cenários.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D3BEC21-D764-43E3-8AC6-5354948A8593}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -18,9 +24,77 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+  <si>
+    <t>Cenário Itapevi</t>
+  </si>
+  <si>
+    <t>Município de (célula C4): Itapevi</t>
+  </si>
+  <si>
+    <t>Matriculados (célula C7): 400</t>
+  </si>
+  <si>
+    <t>Evadidos (célula C8): 31</t>
+  </si>
+  <si>
+    <t>Matriculados (célula C7): 325</t>
+  </si>
+  <si>
+    <t>Cenário Jandira</t>
+  </si>
+  <si>
+    <t>Município de (célula C4): Jandira</t>
+  </si>
+  <si>
+    <t>Matriculados (célula C7): 525</t>
+  </si>
+  <si>
+    <t>Evadidos (célula C8): 32</t>
+  </si>
+  <si>
+    <t>Cenário Osasco</t>
+  </si>
+  <si>
+    <t>Município de (célula C4): Osasco</t>
+  </si>
+  <si>
+    <t>Matriculados (célula C7): 350</t>
+  </si>
+  <si>
+    <t>Evadidos (célula C8): 25</t>
+  </si>
+  <si>
+    <t>Cenário Barueri</t>
+  </si>
+  <si>
+    <t>Município de (célula C4): Barueri</t>
+  </si>
+  <si>
+    <t>Evadidos (célula C8): 35</t>
+  </si>
+  <si>
+    <t>Desempenho de cada Município</t>
+  </si>
+  <si>
+    <t>Alunos</t>
+  </si>
+  <si>
+    <t>Matriculados</t>
+  </si>
+  <si>
+    <t>Evadidos</t>
+  </si>
+  <si>
+    <t>Município de</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +102,44 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -45,12 +147,140 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +560,139 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B1:M9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="12" max="12" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="L1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="L2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="L3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B4" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="L4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="L5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B6" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="12"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="L6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="L7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B8" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="L8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B6:C6"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TAREFA extra CALCULADORA COM MACRO concluída
</commit_message>
<xml_diff>
--- a/Avancado/12 - Teste de Hipóteses - Cenários.xlsx
+++ b/Avancado/12 - Teste de Hipóteses - Cenários.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D3BEC21-D764-43E3-8AC6-5354948A8593}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4FFCC6B-158F-4FA6-A11F-2EBAB3CCE85B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -267,14 +267,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -580,13 +580,13 @@
       </c>
     </row>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
       <c r="L2" s="4" t="s">
         <v>1</v>
       </c>
@@ -595,11 +595,11 @@
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
       <c r="L3" s="4" t="s">
         <v>4</v>
       </c>
@@ -608,13 +608,13 @@
       </c>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
       <c r="L4" s="1" t="s">
         <v>3</v>
       </c>
@@ -623,11 +623,11 @@
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
       <c r="L5" s="3" t="s">
         <v>13</v>
       </c>
@@ -640,9 +640,9 @@
         <v>17</v>
       </c>
       <c r="C6" s="12"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
       <c r="L6" s="4" t="s">
         <v>14</v>
       </c>
@@ -651,13 +651,13 @@
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
       <c r="L7" s="4" t="s">
         <v>2</v>
       </c>
@@ -666,13 +666,13 @@
       </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
       <c r="L8" s="1" t="s">
         <v>15</v>
       </c>
@@ -681,11 +681,11 @@
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>